<commit_message>
Pre-launch review: arithmetic and storyline fixes, expanded credits, glossary deduped, UK spelling, templates reformatted
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_013dXhz1wBJHDaaJTjaDP8MA
</commit_message>
<xml_diff>
--- a/templates/ai-worksheets.xlsx
+++ b/templates/ai-worksheets.xlsx
@@ -18,7 +18,12 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="0"/>
+  <numFmts count="4">
+    <numFmt numFmtId="164" formatCode="#,##0.0"/>
+    <numFmt numFmtId="165" formatCode="0.0%"/>
+    <numFmt numFmtId="166" formatCode="$#,##0"/>
+    <numFmt numFmtId="167" formatCode="$#,##0.00"/>
+  </numFmts>
   <fonts count="5">
     <font>
       <name val="Calibri"/>
@@ -92,7 +97,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="10">
+  <cellXfs count="14">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -101,8 +106,12 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="4" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="4" fontId="0" fillId="3" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="4" fontId="0" fillId="4" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="3" fontId="0" fillId="3" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="164" fontId="0" fillId="3" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="165" fontId="0" fillId="3" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="166" fontId="0" fillId="3" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="167" fontId="0" fillId="3" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="3" fontId="0" fillId="4" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -466,7 +475,7 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
+    <pageSetUpPr fitToPage="1"/>
   </sheetPr>
   <dimension ref="A1:F12"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
@@ -639,6 +648,7 @@
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <pageSetup orientation="landscape" fitToHeight="0" fitToWidth="1"/>
 </worksheet>
 </file>
 
@@ -646,7 +656,7 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
+    <pageSetUpPr fitToPage="1"/>
   </sheetPr>
   <dimension ref="A1:B14"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
@@ -693,7 +703,7 @@
           <t>Hours saved per task (after review time)</t>
         </is>
       </c>
-      <c r="B6" s="8" t="n">
+      <c r="B6" s="9" t="n">
         <v>0.5</v>
       </c>
     </row>
@@ -703,7 +713,7 @@
           <t>Share of freed hours put to new work (0-1)</t>
         </is>
       </c>
-      <c r="B7" s="8" t="n">
+      <c r="B7" s="10" t="n">
         <v>0.7</v>
       </c>
     </row>
@@ -713,7 +723,7 @@
           <t>AI spend this month</t>
         </is>
       </c>
-      <c r="B8" s="8" t="n">
+      <c r="B8" s="11" t="n">
         <v>3000</v>
       </c>
     </row>
@@ -723,7 +733,7 @@
           <t>Average hourly cost of the people</t>
         </is>
       </c>
-      <c r="B9" s="8" t="n">
+      <c r="B9" s="12" t="n">
         <v>60</v>
       </c>
     </row>
@@ -740,7 +750,7 @@
           <t>Realised hours</t>
         </is>
       </c>
-      <c r="B12" s="9">
+      <c r="B12" s="13">
         <f>B5*B6*B7</f>
         <v/>
       </c>
@@ -751,7 +761,7 @@
           <t>AI cost in hours</t>
         </is>
       </c>
-      <c r="B13" s="9">
+      <c r="B13" s="13">
         <f>B8/B9</f>
         <v/>
       </c>
@@ -762,13 +772,14 @@
           <t>Net hours per month</t>
         </is>
       </c>
-      <c r="B14" s="9">
+      <c r="B14" s="13">
         <f>B12-B13</f>
         <v/>
       </c>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <pageSetup orientation="landscape" fitToHeight="0" fitToWidth="1"/>
 </worksheet>
 </file>
 
@@ -776,7 +787,7 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
+    <pageSetUpPr fitToPage="1"/>
   </sheetPr>
   <dimension ref="A1:C15"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
@@ -907,5 +918,6 @@
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <pageSetup orientation="landscape" fitToHeight="0" fitToWidth="1"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Fit Check: four options with configured workflow as the middle ground, fine-tuning last
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_013dXhz1wBJHDaaJTjaDP8MA
</commit_message>
<xml_diff>
--- a/templates/ai-worksheets.xlsx
+++ b/templates/ai-worksheets.xlsx
@@ -475,7 +475,7 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr fitToPage="1"/>
+    <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:F12"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
@@ -648,7 +648,6 @@
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-  <pageSetup orientation="landscape" fitToHeight="0" fitToWidth="1"/>
 </worksheet>
 </file>
 
@@ -656,7 +655,7 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr fitToPage="1"/>
+    <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:B14"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
@@ -779,7 +778,6 @@
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-  <pageSetup orientation="landscape" fitToHeight="0" fitToWidth="1"/>
 </worksheet>
 </file>
 
@@ -787,7 +785,7 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr fitToPage="1"/>
+    <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:C15"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
@@ -831,7 +829,7 @@
       </c>
       <c r="C6" s="4" t="inlineStr">
         <is>
-          <t>Points to (ready-made / adjusted / custom)</t>
+          <t>Points to (ready-made / configured workflow / custom system / fine-tuned)</t>
         </is>
       </c>
     </row>
@@ -847,7 +845,7 @@
     <row r="8">
       <c r="A8" s="6" t="inlineStr">
         <is>
-          <t>Customization: how specific must it be?</t>
+          <t>Customisation: how specific must it be?</t>
         </is>
       </c>
       <c r="B8" s="5" t="inlineStr"/>
@@ -918,6 +916,5 @@
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-  <pageSetup orientation="landscape" fitToHeight="0" fitToWidth="1"/>
 </worksheet>
 </file>
</xml_diff>